<commit_message>
Add Ex4B HW JSON file
</commit_message>
<xml_diff>
--- a/Tewolde_Ex3A_Tables.xlsx
+++ b/Tewolde_Ex3A_Tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\naomitewolde\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C3481EBC-F83B-48F9-A377-9020F32A23F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{96D53DA5-F87C-46CB-BA32-444A09307494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{27C4B28B-AFC7-4415-AA9F-2BDE7A3CF90F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{27C4B28B-AFC7-4415-AA9F-2BDE7A3CF90F}"/>
   </bookViews>
   <sheets>
     <sheet name="Client_Information" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="29" uniqueCount="24">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="36" uniqueCount="31">
   <si>
     <t>Client_ID</t>
   </si>
@@ -113,12 +113,36 @@
   </si>
   <si>
     <t>Special_notes</t>
+  </si>
+  <si>
+    <t>larry</t>
+  </si>
+  <si>
+    <t>pug</t>
+  </si>
+  <si>
+    <t>small</t>
+  </si>
+  <si>
+    <t>allergic to peanuts</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>7 miles</t>
+  </si>
+  <si>
+    <t>1 hour</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -172,12 +196,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -565,10 +591,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7642B86-07CD-4AAF-9038-91DC43AEFCE4}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="20.7265625" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" customWidth="1"/>
     <col min="9" max="9" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -604,6 +631,32 @@
       </c>
       <c r="I2" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="d">
+        <v>2026-01-05</v>
+      </c>
+      <c r="F3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="6">
+        <v>100</v>
+      </c>
+      <c r="I3" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -613,12 +666,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64BE2586-2DE0-41D8-A8A1-E20D19B59FD4}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.1796875" customWidth="1"/>
     <col min="3" max="3" width="11.7265625" customWidth="1"/>
-    <col min="7" max="7" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
@@ -652,6 +705,32 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>